<commit_message>
Report file will be checked in and will be saved in its own folder
</commit_message>
<xml_diff>
--- a/reports/report_2026-03-05.xlsx
+++ b/reports/report_2026-03-05.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S5"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,60 +466,70 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>model_parameters</t>
+          <t>supervisor_temp</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>agent_a_temp</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>agent_b_temp</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>prompt_version</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>classification</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>consensus_reached</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>rounds_used</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>estimated_cost</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>risk_cost</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>risk_flag</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>input_tokens</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>output_tokens</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>ground_truth</t>
         </is>
@@ -528,22 +538,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-05T01:40:42.700163</t>
+          <t>2026-03-05T02:05:50.935003</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20260305_014030_21f19541</t>
+          <t>20260305_020536_1c222e98</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>doc-20260305_014030_21f19541-1</t>
+          <t>doc-20260305_020536_1c222e98-1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>doc_248_vendor_assessment_scores.xlsx</t>
+          <t>C_ 2025 RSCA Procedure - V2.5 with Rating Matrices.docx</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -561,66 +571,70 @@
           <t>anthropic/claude-sonnet-4.5</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>{"supervisor_temp": 0.1, "agent_a_temp": 0.0, "agent_b_temp": 0.0}</t>
-        </is>
+      <c r="H2" t="n">
+        <v>0.1</v>
       </c>
       <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
         <v>1</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>CONFIDENTIAL</t>
         </is>
       </c>
-      <c r="K2" t="n">
-        <v>0.9350000000000001</v>
-      </c>
-      <c r="L2" t="b">
+      <c r="M2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="N2" t="b">
         <v>1</v>
       </c>
-      <c r="M2" t="n">
+      <c r="O2" t="n">
         <v>1</v>
       </c>
-      <c r="N2" t="n">
-        <v>0.0118744</v>
-      </c>
-      <c r="O2" t="n">
-        <v>1.364999999999999</v>
-      </c>
-      <c r="P2" t="inlineStr">
+      <c r="P2" t="n">
+        <v>0.0345044</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1.050000000000001</v>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="Q2" t="n">
-        <v>4280</v>
-      </c>
-      <c r="R2" t="n">
-        <v>1589</v>
-      </c>
-      <c r="S2" t="inlineStr"/>
+      <c r="S2" t="n">
+        <v>16730</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2141</v>
+      </c>
+      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-05T01:42:23.436851</t>
+          <t>2026-03-05T02:07:36.368066</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260305_014153_819ca515</t>
+          <t>20260305_020659_72951757</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>doc-20260305_014153_819ca515-1</t>
+          <t>doc-20260305_020659_72951757-1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>R_sample 3.docx</t>
+          <t>P_NYC Softball Waiver (Independent Contractor).docx</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -638,202 +652,52 @@
           <t>anthropic/claude-sonnet-4.5</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>{"supervisor_temp": 0.1, "agent_a_temp": 0.0, "agent_b_temp": 0.0}</t>
-        </is>
+      <c r="H3" t="n">
+        <v>0.1</v>
       </c>
       <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>CONFIDENTIAL</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="N3" t="b">
         <v>1</v>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>RESTRICTED</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="L3" t="b">
-        <v>1</v>
-      </c>
-      <c r="M3" t="n">
-        <v>1</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.011558</v>
-      </c>
       <c r="O3" t="n">
-        <v>0.08750000000000008</v>
-      </c>
-      <c r="P3" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.0285397</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.20125</v>
+      </c>
+      <c r="R3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="Q3" t="n">
-        <v>3196</v>
-      </c>
-      <c r="R3" t="n">
-        <v>2499</v>
-      </c>
-      <c r="S3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-03-05T01:42:35.227535</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>20260305_014153_819ca515</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>doc-20260305_014153_819ca515-2</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>C_AI_Appropriate_Use_Simplified v1.2.docx</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>google/gemini-3-flash-preview</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>x-ai/grok-4.1-fast</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>anthropic/claude-sonnet-4.5</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>{"supervisor_temp": 0.1, "agent_a_temp": 0.0, "agent_b_temp": 0.0}</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>CONFIDENTIAL</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="L4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.0101987</v>
-      </c>
-      <c r="O4" t="n">
-        <v>1.050000000000001</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="Q4" t="n">
-        <v>3069</v>
-      </c>
-      <c r="R4" t="n">
-        <v>1812</v>
-      </c>
-      <c r="S4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-03-05T01:42:46.941684</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>20260305_014153_819ca515</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>doc-20260305_014153_819ca515-3</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>P_sample.docx</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>google/gemini-3-flash-preview</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>x-ai/grok-4.1-fast</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>anthropic/claude-sonnet-4.5</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>{"supervisor_temp": 0.1, "agent_a_temp": 0.0, "agent_b_temp": 0.0}</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="L5" t="b">
-        <v>1</v>
-      </c>
-      <c r="M5" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.008877599999999999</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.5750000000000005</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="Q5" t="n">
-        <v>2863</v>
-      </c>
-      <c r="R5" t="n">
-        <v>1425</v>
-      </c>
-      <c r="S5" t="inlineStr"/>
+      <c r="S3" t="n">
+        <v>11043</v>
+      </c>
+      <c r="T3" t="n">
+        <v>4268</v>
+      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>